<commit_message>
Excel corrections & AN5397 & imgs
</commit_message>
<xml_diff>
--- a/docs/Kururugi-ESC-sizing.xlsx
+++ b/docs/Kururugi-ESC-sizing.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\binon\Desktop\Kururugi-ESC-Dev-Board\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\binon\Desktop\Kururugi-ESC\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B6FB3AB-61A4-4C9E-A2DB-FE56D7F75C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F82E10B-5E77-4981-893B-E5A7FEFFD2BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="783" xr2:uid="{A7311F5B-F8BB-4208-8795-7C9379CFEF1C}"/>
   </bookViews>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="340">
   <si>
     <t>R1 (kOhm)</t>
   </si>
@@ -518,9 +518,6 @@
   </si>
   <si>
     <t>Min blank time (ns)</t>
-  </si>
-  <si>
-    <t>ADC/OpAmp Isense</t>
   </si>
   <si>
     <t>OpAmp gain</t>
@@ -1281,6 +1278,9 @@
   </si>
   <si>
     <t>ADC Vsense</t>
+  </si>
+  <si>
+    <t>Rshunt &amp; ADC/OpAmp Isense</t>
   </si>
 </sst>
 </file>
@@ -1904,7 +1904,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="177">
+  <cellXfs count="176">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2222,7 +2222,17 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2231,34 +2241,16 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -2267,10 +2259,19 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2336,10 +2337,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2393,6 +2390,12 @@
     </dxf>
     <dxf>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -2731,12 +2734,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -5779,26 +5776,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{E3A51FEF-4642-4801-A998-5B5D5B7E25A4}" name="CAL_Vsense" displayName="CAL_Vsense" ref="B41:H42" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32" tableBorderDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{E3A51FEF-4642-4801-A998-5B5D5B7E25A4}" name="CAL_Vsense" displayName="CAL_Vsense" ref="B41:H42" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34" tableBorderDxfId="33">
   <autoFilter ref="B41:H42" xr:uid="{E3A51FEF-4642-4801-A998-5B5D5B7E25A4}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{72CE8DA8-6563-4322-AABC-36ACF43055CB}" name="Rbot (Ω)" dataDxfId="30">
+    <tableColumn id="1" xr3:uid="{72CE8DA8-6563-4322-AABC-36ACF43055CB}" name="Rbot (Ω)" dataDxfId="32">
       <calculatedColumnFormula>HMI!U17</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{24747B59-61B7-4C72-90DC-263488210056}" name="Rbot/Rtop" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{DDE3289D-88E0-4C7D-87FD-D3D69E79F10D}" name="Rtop (Ω)" dataDxfId="28">
+    <tableColumn id="2" xr3:uid="{24747B59-61B7-4C72-90DC-263488210056}" name="Rbot/Rtop" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{DDE3289D-88E0-4C7D-87FD-D3D69E79F10D}" name="Rtop (Ω)" dataDxfId="30">
       <calculatedColumnFormula>HMI!U18</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{6958CE2B-2C13-409D-93AE-44178BFFDA66}" name="Rth (Ω)" dataDxfId="27">
+    <tableColumn id="4" xr3:uid="{6958CE2B-2C13-409D-93AE-44178BFFDA66}" name="Rth (Ω)" dataDxfId="29">
       <calculatedColumnFormula>CAL_Vsense[[#This Row],[Rtop (Ω)]]*CAL_Vsense[[#This Row],[Rbot (Ω)]]/(CAL_Vsense[[#This Row],[Rbot (Ω)]]+CAL_Vsense[[#This Row],[Rtop (Ω)]])+Radc</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{11134CB2-C2E0-49B7-9A9A-CCA3E473CAA8}" name="Iadc (mA)" dataDxfId="26">
+    <tableColumn id="5" xr3:uid="{11134CB2-C2E0-49B7-9A9A-CCA3E473CAA8}" name="Iadc (mA)" dataDxfId="28">
       <calculatedColumnFormula array="1">DB_ADC[Vref,adc (V)]/CAL_Vsense[[#This Row],[Rth (Ω)]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{C0D5F77C-6884-4436-8011-5E3C9BAF9068}" name="R_CinToAdc (Ω)" dataDxfId="25">
+    <tableColumn id="6" xr3:uid="{C0D5F77C-6884-4436-8011-5E3C9BAF9068}" name="R_CinToAdc (Ω)" dataDxfId="27">
       <calculatedColumnFormula array="1">HMI!U21*#REF!/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{33243AAC-B51F-4185-98EF-90101F594D74}" name="S*RCint (ps)" dataDxfId="24">
+    <tableColumn id="7" xr3:uid="{33243AAC-B51F-4185-98EF-90101F594D74}" name="S*RCint (ps)" dataDxfId="26">
       <calculatedColumnFormula>HMI!U22*CAL_Vsense[[#This Row],[R_CinToAdc (Ω)]]*HMI!U21</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5807,25 +5804,25 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E81DD96E-7100-4CD1-9FCC-4539084BC6B8}" name="Table8" displayName="Table8" ref="B3:G14" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" headerRowBorderDxfId="22" tableBorderDxfId="20" totalsRowBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E81DD96E-7100-4CD1-9FCC-4539084BC6B8}" name="Table8" displayName="Table8" ref="B3:G14" totalsRowShown="0" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24" tableBorderDxfId="22" totalsRowBorderDxfId="21">
   <autoFilter ref="B3:G14" xr:uid="{E81DD96E-7100-4CD1-9FCC-4539084BC6B8}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{11F74BC1-EDA3-4B09-9543-C91ACD28F6D6}" name="Rshunt (µOhm)" dataDxfId="18">
+    <tableColumn id="1" xr3:uid="{11F74BC1-EDA3-4B09-9543-C91ACD28F6D6}" name="Rshunt (µOhm)" dataDxfId="20">
       <calculatedColumnFormula>B3+100</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F22209D4-D5F7-4A24-A22E-BCB1F60E1A02}" name="Disspated power (W)" dataDxfId="17">
+    <tableColumn id="2" xr3:uid="{F22209D4-D5F7-4A24-A22E-BCB1F60E1A02}" name="Disspated power (W)" dataDxfId="19">
       <calculatedColumnFormula>B4*$J$5*$J$5/1000/1000*$J$3/100</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{D529F738-8D82-4F6B-AFA8-BE5DBAB5E958}" name="Voltage drop spike amp (V)" dataDxfId="16">
+    <tableColumn id="3" xr3:uid="{D529F738-8D82-4F6B-AFA8-BE5DBAB5E958}" name="Voltage drop spike amp (V)" dataDxfId="18">
       <calculatedColumnFormula>$J$6*B4/1000*$J$12/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DA16F6C7-9239-4007-9C54-6D51F73E46DA}" name="Voltage drop max amp (V)" dataDxfId="15">
+    <tableColumn id="4" xr3:uid="{DA16F6C7-9239-4007-9C54-6D51F73E46DA}" name="Voltage drop max amp (V)" dataDxfId="17">
       <calculatedColumnFormula>$J$5*B4/1000*$J$12/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{B27B3633-2D8E-48A1-A695-660FCB0A39C1}" name="Voltage drop typ amp (V)2" dataDxfId="14">
+    <tableColumn id="6" xr3:uid="{B27B3633-2D8E-48A1-A695-660FCB0A39C1}" name="Voltage drop typ amp (V)2" dataDxfId="16">
       <calculatedColumnFormula>$J$4*B4/1000*$J$12/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{F4370240-49C3-4C3D-A378-B3808740E62D}" name="mA/step" dataDxfId="13">
+    <tableColumn id="5" xr3:uid="{F4370240-49C3-4C3D-A378-B3808740E62D}" name="mA/step" dataDxfId="15">
       <calculatedColumnFormula>$J$6/(D4/1000*$J$10/$J$8)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5860,12 +5857,12 @@
     <tableColumn id="17" xr3:uid="{8828BB6B-7ABC-4BA6-9E1B-5C5BE5105F08}" name="Iph typ (A)"/>
     <tableColumn id="18" xr3:uid="{1F68324A-F399-4C91-BE2D-EFEF49ED6790}" name="ToF Iph typ (%)"/>
     <tableColumn id="15" xr3:uid="{5ED528D3-58D8-4741-86F9-6B25ECFBAFAE}" name="Iph max (A@Xs)"/>
-    <tableColumn id="19" xr3:uid="{305A20A8-F4F6-4F6B-BAC2-2A71E7628C5B}" name="ToF Iph max (%)" dataDxfId="35">
+    <tableColumn id="19" xr3:uid="{305A20A8-F4F6-4F6B-BAC2-2A71E7628C5B}" name="ToF Iph max (%)" dataDxfId="14">
       <calculatedColumnFormula>100-DB_limits[[#This Row],[ToF Iph typ (%)]]-DB_limits[[#This Row],[ToF Iph spike (%)]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="16" xr3:uid="{4D711E23-0E80-41C8-A566-2B43E0C79E4C}" name="Iph spike (A@Xms)"/>
     <tableColumn id="20" xr3:uid="{0DE3AE78-D822-41D8-B4E1-38C2CE21BE19}" name="ToF Iph spike (%)"/>
-    <tableColumn id="21" xr3:uid="{0DD4A4A7-CFA4-4B62-89A9-A58896065868}" name="Iph mean (A)" dataDxfId="34">
+    <tableColumn id="21" xr3:uid="{0DD4A4A7-CFA4-4B62-89A9-A58896065868}" name="Iph mean (A)" dataDxfId="13">
       <calculatedColumnFormula>DB_limits[[#This Row],[Iph typ (A)]]*DB_limits[[#This Row],[ToF Iph typ (%)]]%+DB_limits[[#This Row],[Iph max (A@Xs)]]*DB_limits[[#This Row],[ToF Iph max (%)]]%+DB_limits[[#This Row],[Iph spike (A@Xms)]]*DB_limits[[#This Row],[ToF Iph spike (%)]]%</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="24" xr3:uid="{47619F70-8E0D-4CA7-A6D9-A367CF759D25}" name="Termistors"/>
@@ -6325,95 +6322,93 @@
   <sheetData>
     <row r="1" spans="2:21" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B2" s="138" t="s">
+      <c r="B2" s="142" t="s">
         <v>117</v>
       </c>
-      <c r="C2" s="139"/>
-      <c r="E2" s="138" t="s">
-        <v>145</v>
-      </c>
-      <c r="F2" s="139"/>
-      <c r="H2" s="138" t="s">
+      <c r="C2" s="143"/>
+      <c r="E2" s="142" t="s">
+        <v>144</v>
+      </c>
+      <c r="F2" s="143"/>
+      <c r="H2" s="142" t="s">
         <v>102</v>
       </c>
-      <c r="I2" s="139"/>
-      <c r="K2" s="138" t="s">
-        <v>226</v>
-      </c>
-      <c r="L2" s="139"/>
-      <c r="N2" s="138" t="s">
-        <v>255</v>
-      </c>
-      <c r="O2" s="139"/>
-      <c r="Q2" s="138" t="s">
+      <c r="I2" s="143"/>
+      <c r="K2" s="140" t="s">
+        <v>339</v>
+      </c>
+      <c r="L2" s="141"/>
+      <c r="N2" s="142" t="s">
+        <v>254</v>
+      </c>
+      <c r="O2" s="143"/>
+      <c r="Q2" s="142" t="s">
+        <v>323</v>
+      </c>
+      <c r="R2" s="143"/>
+      <c r="T2" s="149"/>
+      <c r="U2" s="149"/>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.35">
+      <c r="B3" s="144" t="s">
+        <v>200</v>
+      </c>
+      <c r="C3" s="145"/>
+      <c r="D3" s="113"/>
+      <c r="E3" s="151" t="s">
+        <v>203</v>
+      </c>
+      <c r="F3" s="152"/>
+      <c r="H3" s="144" t="s">
+        <v>201</v>
+      </c>
+      <c r="I3" s="145"/>
+      <c r="K3" s="138" t="s">
+        <v>113</v>
+      </c>
+      <c r="L3" s="139"/>
+      <c r="N3" s="144" t="s">
+        <v>131</v>
+      </c>
+      <c r="O3" s="145"/>
+      <c r="Q3" s="144" t="s">
+        <v>131</v>
+      </c>
+      <c r="R3" s="145"/>
+      <c r="T3" s="150"/>
+      <c r="U3" s="150"/>
+    </row>
+    <row r="4" spans="2:21" x14ac:dyDescent="0.35">
+      <c r="B4" s="146" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="147"/>
+      <c r="E4" s="144" t="s">
+        <v>131</v>
+      </c>
+      <c r="F4" s="145"/>
+      <c r="H4" s="146" t="s">
+        <v>202</v>
+      </c>
+      <c r="I4" s="147"/>
+      <c r="K4" s="151" t="s">
+        <v>132</v>
+      </c>
+      <c r="L4" s="152"/>
+      <c r="N4" s="117" t="s">
+        <v>260</v>
+      </c>
+      <c r="O4" s="61" t="s">
+        <v>329</v>
+      </c>
+      <c r="Q4" s="117" t="s">
         <v>324</v>
       </c>
-      <c r="R2" s="139"/>
-      <c r="T2" s="151"/>
-      <c r="U2" s="151"/>
-    </row>
-    <row r="3" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B3" s="142" t="s">
-        <v>201</v>
-      </c>
-      <c r="C3" s="143"/>
-      <c r="D3" s="113"/>
-      <c r="E3" s="140" t="s">
-        <v>204</v>
-      </c>
-      <c r="F3" s="141"/>
-      <c r="H3" s="142" t="s">
-        <v>202</v>
-      </c>
-      <c r="I3" s="143"/>
-      <c r="K3" s="142" t="s">
-        <v>131</v>
-      </c>
-      <c r="L3" s="143"/>
-      <c r="N3" s="142" t="s">
-        <v>131</v>
-      </c>
-      <c r="O3" s="143"/>
-      <c r="Q3" s="142" t="s">
-        <v>131</v>
-      </c>
-      <c r="R3" s="143"/>
-      <c r="T3" s="137"/>
-      <c r="U3" s="137"/>
-    </row>
-    <row r="4" spans="2:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="152" t="s">
-        <v>118</v>
-      </c>
-      <c r="C4" s="153"/>
-      <c r="E4" s="142" t="s">
-        <v>131</v>
-      </c>
-      <c r="F4" s="143"/>
-      <c r="H4" s="152" t="s">
-        <v>203</v>
-      </c>
-      <c r="I4" s="153"/>
-      <c r="K4" s="118" t="s">
-        <v>243</v>
-      </c>
-      <c r="L4" s="119">
-        <v>850</v>
-      </c>
-      <c r="N4" s="117" t="s">
-        <v>261</v>
-      </c>
-      <c r="O4" s="61" t="s">
-        <v>330</v>
-      </c>
-      <c r="Q4" s="117" t="s">
-        <v>325</v>
-      </c>
       <c r="R4" s="61" t="s">
-        <v>332</v>
-      </c>
-      <c r="T4" s="150"/>
-      <c r="U4" s="150"/>
+        <v>331</v>
+      </c>
+      <c r="T4" s="148"/>
+      <c r="U4" s="148"/>
     </row>
     <row r="5" spans="2:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="70" t="str">
@@ -6438,6 +6433,14 @@
         <f>_xlfn.XLOOKUP(H4, DB_Mostfet[Part], DB_Mostfet[Vds (V)])</f>
         <v>60</v>
       </c>
+      <c r="K5" s="70" t="str">
+        <f>DB_ADC[[#Headers],[Vmax (V)]]</f>
+        <v>Vmax (V)</v>
+      </c>
+      <c r="L5" s="61">
+        <f>_xlfn.XLOOKUP($K$4, DB_ADC[Name], DB_ADC[Vmax (V)])</f>
+        <v>3.5999999999999996</v>
+      </c>
       <c r="N5" s="70" t="str">
         <f>DB_R[[#Headers],[Prated@70°C (mW)]]</f>
         <v>Prated@70°C (mW)</v>
@@ -6447,10 +6450,10 @@
         <v>65</v>
       </c>
       <c r="Q5" s="117" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R5" s="61" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="U5" s="93"/>
     </row>
@@ -6471,20 +6474,20 @@
         <f>_xlfn.XLOOKUP(H4, DB_Mostfet[Part], DB_Mostfet[Qg,typ @ 10V (nC)])</f>
         <v>41</v>
       </c>
-      <c r="K6" s="144" t="s">
-        <v>140</v>
-      </c>
-      <c r="L6" s="145"/>
+      <c r="K6" s="138" t="s">
+        <v>131</v>
+      </c>
+      <c r="L6" s="139"/>
       <c r="N6" s="117" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="O6" s="61" t="s">
-        <v>331</v>
-      </c>
-      <c r="Q6" s="146" t="s">
+        <v>330</v>
+      </c>
+      <c r="Q6" s="138" t="s">
         <v>130</v>
       </c>
-      <c r="R6" s="147"/>
+      <c r="R6" s="139"/>
       <c r="U6" s="93"/>
     </row>
     <row r="7" spans="2:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -6496,10 +6499,10 @@
         <f>_xlfn.XLOOKUP(B4,DB_limits[Name],DB_limits[Fmax (kHz)])</f>
         <v>64</v>
       </c>
-      <c r="E7" s="138" t="s">
-        <v>225</v>
-      </c>
-      <c r="F7" s="139"/>
+      <c r="E7" s="142" t="s">
+        <v>224</v>
+      </c>
+      <c r="F7" s="143"/>
       <c r="H7" s="70" t="str">
         <f>DB_Mostfet[[#Headers],[Qg,typ,sync @ 10V (nC)]] &amp;  " (not used)"</f>
         <v>Qg,typ,sync @ 10V (nC) (not used)</v>
@@ -6508,10 +6511,12 @@
         <f>_xlfn.XLOOKUP(H4, DB_Mostfet[Part], DB_Mostfet[Qg,typ,sync @ 10V (nC)])</f>
         <v>X</v>
       </c>
-      <c r="K7" s="146" t="s">
-        <v>113</v>
-      </c>
-      <c r="L7" s="147"/>
+      <c r="K7" s="117" t="s">
+        <v>242</v>
+      </c>
+      <c r="L7" s="61">
+        <v>500</v>
+      </c>
       <c r="N7" s="121" t="str">
         <f>N5</f>
         <v>Prated@70°C (mW)</v>
@@ -6539,10 +6544,10 @@
         <f>_xlfn.XLOOKUP($B$4, DB_limits[Name], DB_limits[Vbat,min (V)])</f>
         <v>14</v>
       </c>
-      <c r="E8" s="148" t="s">
-        <v>207</v>
-      </c>
-      <c r="F8" s="149"/>
+      <c r="E8" s="153" t="s">
+        <v>206</v>
+      </c>
+      <c r="F8" s="154"/>
       <c r="H8" s="70" t="str">
         <f>DB_Mostfet[[#Headers],[Rds,on@10V typ(mΩ)]] &amp;  " (not used)"</f>
         <v>Rds,on@10V typ(mΩ) (not used)</v>
@@ -6551,10 +6556,12 @@
         <f>_xlfn.XLOOKUP(H4, DB_Mostfet[Part], DB_Mostfet[Rds,on@10V typ(mΩ)])</f>
         <v>1.8</v>
       </c>
-      <c r="K8" s="152" t="s">
-        <v>132</v>
-      </c>
-      <c r="L8" s="153"/>
+      <c r="K8" s="117" t="s">
+        <v>127</v>
+      </c>
+      <c r="L8" s="61">
+        <v>12</v>
+      </c>
       <c r="Q8" s="73" t="str">
         <f>CAL_Vbat!G13</f>
         <v>Vbat,adc,typ (V)</v>
@@ -6582,18 +6589,16 @@
         <f>_xlfn.XLOOKUP(H4, DB_Mostfet[Part], DB_Mostfet[Rds,on@10V max (mΩ)])</f>
         <v>2.2000000000000002</v>
       </c>
-      <c r="K9" s="70" t="str">
-        <f>DB_ADC[[#Headers],[Vmax (V)]]</f>
-        <v>Vmax (V)</v>
+      <c r="K9" s="117" t="s">
+        <v>277</v>
       </c>
       <c r="L9" s="61">
-        <f>_xlfn.XLOOKUP($K$8, DB_ADC[Name], DB_ADC[Vmax (V)])</f>
-        <v>3.5999999999999996</v>
-      </c>
-      <c r="N9" s="144" t="s">
-        <v>339</v>
-      </c>
-      <c r="O9" s="145"/>
+        <v>2.5</v>
+      </c>
+      <c r="N9" s="140" t="s">
+        <v>338</v>
+      </c>
+      <c r="O9" s="141"/>
       <c r="Q9" s="87" t="str">
         <f>CAL_Vbat!G20</f>
         <v>Rbat,adc,thev (Ω)</v>
@@ -6614,10 +6619,10 @@
         <f>_xlfn.XLOOKUP($B$4, DB_limits[Name], DB_limits[Vbat spike (V) @ run])</f>
         <v>32</v>
       </c>
-      <c r="E10" s="144" t="s">
-        <v>216</v>
-      </c>
-      <c r="F10" s="145"/>
+      <c r="E10" s="140" t="s">
+        <v>215</v>
+      </c>
+      <c r="F10" s="141"/>
       <c r="H10" s="70" t="str">
         <f>DB_Mostfet[[#Headers],[Id @ Tc&gt;70°C (A)]]</f>
         <v>Id @ Tc&gt;70°C (A)</v>
@@ -6626,14 +6631,16 @@
         <f>_xlfn.XLOOKUP(H4, DB_Mostfet[Part], DB_Mostfet[Id @ Tc&gt;70°C (A)])</f>
         <v>100</v>
       </c>
-      <c r="K10" s="146" t="s">
-        <v>131</v>
-      </c>
-      <c r="L10" s="147"/>
-      <c r="N10" s="146" t="s">
+      <c r="K10" s="117" t="s">
+        <v>140</v>
+      </c>
+      <c r="L10" s="61">
+        <v>64</v>
+      </c>
+      <c r="N10" s="138" t="s">
         <v>113</v>
       </c>
-      <c r="O10" s="147"/>
+      <c r="O10" s="139"/>
       <c r="R10" s="93"/>
       <c r="U10" s="93"/>
     </row>
@@ -6646,10 +6653,10 @@
         <f>_xlfn.XLOOKUP($B$4, DB_limits[Name], DB_limits[Vbat spike (V) @ disarm])</f>
         <v>45</v>
       </c>
-      <c r="E11" s="146" t="s">
+      <c r="E11" s="138" t="s">
         <v>131</v>
       </c>
-      <c r="F11" s="147"/>
+      <c r="F11" s="139"/>
       <c r="H11" s="70" t="str">
         <f>DB_Mostfet[[#Headers],[Id @ Ta&gt;70°C (A)]]</f>
         <v>Id @ Ta&gt;70°C (A)</v>
@@ -6658,16 +6665,14 @@
         <f>_xlfn.XLOOKUP(H4, DB_Mostfet[Part], DB_Mostfet[Id @ Ta&gt;70°C (A)])</f>
         <v>(est ~21A)</v>
       </c>
-      <c r="K11" s="117" t="s">
-        <v>127</v>
-      </c>
-      <c r="L11" s="61">
-        <v>12</v>
-      </c>
-      <c r="N11" s="140" t="s">
+      <c r="K11" s="138" t="s">
+        <v>130</v>
+      </c>
+      <c r="L11" s="139"/>
+      <c r="N11" s="151" t="s">
         <v>132</v>
       </c>
-      <c r="O11" s="141"/>
+      <c r="O11" s="152"/>
       <c r="R11" s="93"/>
       <c r="U11" s="93"/>
     </row>
@@ -6681,7 +6686,7 @@
         <v>35</v>
       </c>
       <c r="E12" s="118" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F12" s="119">
         <v>10</v>
@@ -6694,11 +6699,12 @@
         <f>_xlfn.XLOOKUP(H4, DB_Mostfet[Part], DB_Mostfet[Size (mm)])</f>
         <v>5x6</v>
       </c>
-      <c r="K12" s="117" t="s">
-        <v>278</v>
-      </c>
-      <c r="L12" s="61">
-        <v>2.5</v>
+      <c r="K12" s="73" t="s">
+        <v>293</v>
+      </c>
+      <c r="L12" s="78">
+        <f>(L8+L9+0.5)*_xlfn.XLOOKUP(K4,DB_ADC[Name],DB_ADC[Tadc,clock (ns)])</f>
+        <v>250.00000000000003</v>
       </c>
       <c r="N12" s="70" t="str">
         <f>DB_ADC[[#Headers],[Csamp (pF)]]</f>
@@ -6730,11 +6736,13 @@
         <f>_xlfn.XLOOKUP(H4, DB_Mostfet[Part], DB_Mostfet[JLCPBC stock])</f>
         <v>Yes</v>
       </c>
-      <c r="K13" s="117" t="s">
-        <v>141</v>
-      </c>
-      <c r="L13" s="61">
-        <v>64</v>
+      <c r="K13" s="124" t="str">
+        <f>CAL_Rshunt!G22</f>
+        <v>Vshunt,amp,spike (V)</v>
+      </c>
+      <c r="L13" s="128">
+        <f>CAL_Rshunt!H22</f>
+        <v>1.6</v>
       </c>
       <c r="N13" s="70" t="str">
         <f>DB_ADC[[#Headers],[Cpad (pF)]]</f>
@@ -6757,22 +6765,26 @@
         <f>_xlfn.XLOOKUP($B$4, DB_limits[Name], DB_limits[Iph typ (A)])</f>
         <v>12.5</v>
       </c>
-      <c r="E14" s="144" t="s">
-        <v>253</v>
-      </c>
-      <c r="F14" s="145"/>
-      <c r="H14" s="142" t="s">
+      <c r="E14" s="140" t="s">
+        <v>252</v>
+      </c>
+      <c r="F14" s="141"/>
+      <c r="H14" s="144" t="s">
         <v>130</v>
       </c>
-      <c r="I14" s="143"/>
-      <c r="K14" s="146" t="s">
-        <v>130</v>
-      </c>
-      <c r="L14" s="147"/>
-      <c r="N14" s="146" t="s">
+      <c r="I14" s="145"/>
+      <c r="K14" s="124" t="str">
+        <f>CAL_Rshunt!J6</f>
+        <v>ΔIlsb (mA/bit)</v>
+      </c>
+      <c r="L14" s="128">
+        <f>CAL_Rshunt!K6</f>
+        <v>25.183150183150182</v>
+      </c>
+      <c r="N14" s="138" t="s">
         <v>131</v>
       </c>
-      <c r="O14" s="147"/>
+      <c r="O14" s="139"/>
       <c r="R14" s="94"/>
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.35">
@@ -6784,10 +6796,10 @@
         <f>_xlfn.XLOOKUP($B$4, DB_limits[Name], DB_limits[Iph max (A@Xs)])</f>
         <v>20</v>
       </c>
-      <c r="E15" s="146" t="s">
+      <c r="E15" s="138" t="s">
         <v>131</v>
       </c>
-      <c r="F15" s="147"/>
+      <c r="F15" s="139"/>
       <c r="H15" s="73" t="str">
         <f>CAL_Fets!G28</f>
         <v>Ptot,typ (mW)</v>
@@ -6796,12 +6808,13 @@
         <f>CAL_Fets!H28</f>
         <v>1667.2220807894741</v>
       </c>
-      <c r="K15" s="73" t="s">
-        <v>294</v>
+      <c r="K15" s="73" t="str">
+        <f>CAL_Rshunt!J14</f>
+        <v>Pshunt,mean (mW)</v>
       </c>
       <c r="L15" s="78">
-        <f>(L11+L12+0.5)*_xlfn.XLOOKUP(K8,DB_ADC[Name],DB_ADC[Tadc,clock (ns)])</f>
-        <v>250.00000000000003</v>
+        <f>CAL_Rshunt!K14</f>
+        <v>49.961707500000017</v>
       </c>
       <c r="N15" s="117" t="s">
         <v>127</v>
@@ -6822,7 +6835,7 @@
         <v>50</v>
       </c>
       <c r="E16" s="134" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F16" s="136">
         <v>60</v>
@@ -6835,16 +6848,16 @@
         <f>CAL_Fets!H29</f>
         <v>3145.7629473684219</v>
       </c>
-      <c r="K16" s="124" t="str">
-        <f>CAL_Rshunt!G22</f>
-        <v>Vshunt,amp,spike (V)</v>
-      </c>
-      <c r="L16" s="128">
-        <f>CAL_Rshunt!H22</f>
-        <v>2.72</v>
+      <c r="K16" s="126" t="str">
+        <f>CAL_Rshunt!J22</f>
+        <v>Pshunt,max (mW@Xs)</v>
+      </c>
+      <c r="L16" s="129">
+        <f>CAL_Rshunt!K22</f>
+        <v>120</v>
       </c>
       <c r="N16" s="117" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="O16" s="61">
         <v>2.5</v>
@@ -6864,21 +6877,13 @@
         <v>12.905000000000001</v>
       </c>
       <c r="E17" s="134" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F17" s="136">
         <v>30</v>
       </c>
-      <c r="K17" s="124" t="str">
-        <f>CAL_Rshunt!J6</f>
-        <v>ΔIlsb (mA/bit)</v>
-      </c>
-      <c r="L17" s="128">
-        <f>CAL_Rshunt!K6</f>
-        <v>14.813617754794226</v>
-      </c>
       <c r="N17" s="130" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="O17" s="131">
         <v>5</v>
@@ -6897,47 +6902,31 @@
         <v>1 (at a FET)</v>
       </c>
       <c r="E18" s="134" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F18" s="135">
         <v>3</v>
       </c>
-      <c r="K18" s="73" t="str">
-        <f>CAL_Rshunt!J14</f>
-        <v>Pshunt,mean (mW)</v>
-      </c>
-      <c r="L18" s="78">
-        <f>CAL_Rshunt!K14</f>
-        <v>84.934902750000006</v>
-      </c>
-      <c r="N18" s="146" t="s">
+      <c r="N18" s="138" t="s">
         <v>130</v>
       </c>
-      <c r="O18" s="147"/>
+      <c r="O18" s="139"/>
       <c r="R18" s="92"/>
       <c r="U18" s="93"/>
     </row>
-    <row r="19" spans="2:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="146" t="s">
+    <row r="19" spans="2:21" x14ac:dyDescent="0.35">
+      <c r="B19" s="138" t="s">
         <v>131</v>
       </c>
-      <c r="C19" s="147"/>
+      <c r="C19" s="139"/>
       <c r="E19" s="117" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F19" s="61">
         <v>3.3</v>
       </c>
-      <c r="K19" s="126" t="str">
-        <f>CAL_Rshunt!J22</f>
-        <v>Pshunt,max (mW@Xs)</v>
-      </c>
-      <c r="L19" s="129">
-        <f>CAL_Rshunt!K22</f>
-        <v>204</v>
-      </c>
       <c r="N19" s="73" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="O19" s="78">
         <f>(O15+O16+0.5)*_xlfn.XLOOKUP(N11,DB_ADC[Name],DB_ADC[Tadc,clock (ns)])</f>
@@ -6953,10 +6942,10 @@
       <c r="C20" s="61">
         <v>480</v>
       </c>
-      <c r="E20" s="146" t="s">
+      <c r="E20" s="138" t="s">
         <v>130</v>
       </c>
-      <c r="F20" s="147"/>
+      <c r="F20" s="139"/>
       <c r="N20" s="73" t="str">
         <f>'CAL_Rv1-2'!G5</f>
         <v>Rv1,th (Ω)</v>
@@ -6970,7 +6959,7 @@
     </row>
     <row r="21" spans="2:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B21" s="118" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C21" s="119">
         <v>300</v>
@@ -7032,8 +7021,8 @@
         <v>3.1818181818181817</v>
       </c>
       <c r="R23" s="91"/>
-      <c r="T23" s="137"/>
-      <c r="U23" s="137"/>
+      <c r="T23" s="150"/>
+      <c r="U23" s="150"/>
     </row>
     <row r="24" spans="2:21" x14ac:dyDescent="0.35">
       <c r="E24" s="73" t="str">
@@ -7116,21 +7105,21 @@
       <c r="U28" s="94"/>
     </row>
     <row r="29" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="E29" s="144" t="s">
-        <v>230</v>
-      </c>
-      <c r="F29" s="145"/>
+      <c r="E29" s="140" t="s">
+        <v>229</v>
+      </c>
+      <c r="F29" s="141"/>
       <c r="N29" s="122" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="O29" s="123"/>
       <c r="U29" s="91"/>
     </row>
     <row r="30" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="E30" s="146" t="s">
+      <c r="E30" s="138" t="s">
         <v>131</v>
       </c>
-      <c r="F30" s="147"/>
+      <c r="F30" s="139"/>
       <c r="N30" s="115" t="s">
         <v>131</v>
       </c>
@@ -7138,13 +7127,13 @@
     </row>
     <row r="31" spans="2:21" x14ac:dyDescent="0.35">
       <c r="E31" s="117" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F31" s="61">
         <v>3.3</v>
       </c>
       <c r="N31" s="117" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="O31" s="61">
         <v>100</v>
@@ -7152,13 +7141,13 @@
     </row>
     <row r="32" spans="2:21" x14ac:dyDescent="0.35">
       <c r="E32" s="117" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F32" s="61">
         <v>10</v>
       </c>
       <c r="N32" s="134" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="O32" s="136">
         <v>40</v>
@@ -7166,25 +7155,25 @@
     </row>
     <row r="33" spans="5:15" x14ac:dyDescent="0.35">
       <c r="E33" s="134" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F33" s="135">
         <v>1.5</v>
       </c>
       <c r="N33" s="134" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="O33" s="136">
         <v>12</v>
       </c>
     </row>
     <row r="34" spans="5:15" x14ac:dyDescent="0.35">
-      <c r="E34" s="146" t="s">
+      <c r="E34" s="138" t="s">
         <v>130</v>
       </c>
-      <c r="F34" s="147"/>
+      <c r="F34" s="139"/>
       <c r="N34" s="134" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="O34" s="136">
         <v>5</v>
@@ -7268,7 +7257,7 @@
         <v>40.383359999999996</v>
       </c>
       <c r="N39" s="67" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="40" spans="5:15" x14ac:dyDescent="0.35">
@@ -7281,7 +7270,7 @@
         <v>27.360304480749178</v>
       </c>
       <c r="N40" s="67" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="41" spans="5:15" x14ac:dyDescent="0.35">
@@ -7305,33 +7294,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="42">
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="Q2:R2"/>
-    <mergeCell ref="Q3:R3"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="T4:U4"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="T3:U3"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="N18:O18"/>
+  <mergeCells count="40">
     <mergeCell ref="T23:U23"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>
@@ -7345,9 +7308,33 @@
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="K6:L6"/>
-    <mergeCell ref="K7:L7"/>
     <mergeCell ref="N14:O14"/>
     <mergeCell ref="E8:F8"/>
+    <mergeCell ref="T4:U4"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="T3:U3"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="Q2:R2"/>
+    <mergeCell ref="Q3:R3"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="K4:L4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7365,7 +7352,7 @@
           <x14:formula1>
             <xm:f>DB_ADC!$A$2:$A$21</xm:f>
           </x14:formula1>
-          <xm:sqref>N11 T4 K8</xm:sqref>
+          <xm:sqref>N11 T4 K4</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{85D05625-9851-4F66-A584-AE65C6830A4B}">
           <x14:formula1>
@@ -7434,7 +7421,7 @@
         <v>126</v>
       </c>
       <c r="C1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D1" t="s">
         <v>101</v>
@@ -7458,46 +7445,46 @@
         <v>125</v>
       </c>
       <c r="K1" t="s">
+        <v>266</v>
+      </c>
+      <c r="L1" t="s">
         <v>267</v>
       </c>
-      <c r="L1" t="s">
-        <v>268</v>
-      </c>
       <c r="M1" t="s">
+        <v>192</v>
+      </c>
+      <c r="N1" t="s">
+        <v>194</v>
+      </c>
+      <c r="O1" t="s">
+        <v>191</v>
+      </c>
+      <c r="P1" t="s">
         <v>193</v>
       </c>
-      <c r="N1" t="s">
-        <v>195</v>
-      </c>
-      <c r="O1" t="s">
-        <v>192</v>
-      </c>
-      <c r="P1" t="s">
-        <v>194</v>
-      </c>
       <c r="Q1" t="s">
+        <v>154</v>
+      </c>
+      <c r="R1" t="s">
+        <v>159</v>
+      </c>
+      <c r="S1" t="s">
         <v>155</v>
       </c>
-      <c r="R1" t="s">
+      <c r="T1" t="s">
         <v>160</v>
       </c>
-      <c r="S1" t="s">
+      <c r="U1" t="s">
         <v>156</v>
       </c>
-      <c r="T1" t="s">
+      <c r="V1" t="s">
         <v>161</v>
       </c>
-      <c r="U1" t="s">
-        <v>157</v>
-      </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>162</v>
       </c>
-      <c r="W1" t="s">
-        <v>163</v>
-      </c>
       <c r="X1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
@@ -7575,12 +7562,12 @@
         <v>12.905000000000001</v>
       </c>
       <c r="X2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B3">
         <v>6</v>
@@ -7653,12 +7640,12 @@
         <v>12.905000000000001</v>
       </c>
       <c r="X3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -7731,12 +7718,12 @@
         <v>14.625</v>
       </c>
       <c r="X4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B5">
         <v>6</v>
@@ -7809,7 +7796,7 @@
         <v>12.905000000000001</v>
       </c>
       <c r="X5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.35">
@@ -7887,12 +7874,12 @@
         <v>16.850000000000001</v>
       </c>
       <c r="X6" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B7">
         <v>6</v>
@@ -7965,7 +7952,7 @@
         <v>14.625</v>
       </c>
       <c r="X7" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -8001,10 +7988,10 @@
         <v>98</v>
       </c>
       <c r="C1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E1" t="s">
         <v>100</v>
@@ -8013,27 +8000,27 @@
         <v>99</v>
       </c>
       <c r="G1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H1" t="s">
+        <v>149</v>
+      </c>
+      <c r="I1" t="s">
         <v>150</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>151</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>152</v>
       </c>
-      <c r="K1" t="s">
-        <v>153</v>
-      </c>
       <c r="L1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B2">
         <v>6</v>
@@ -8125,28 +8112,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D1" t="s">
+        <v>337</v>
+      </c>
+      <c r="E1" t="s">
         <v>257</v>
       </c>
-      <c r="B1" t="s">
-        <v>211</v>
-      </c>
-      <c r="C1" t="s">
-        <v>227</v>
-      </c>
-      <c r="D1" t="s">
-        <v>338</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>258</v>
-      </c>
-      <c r="F1" t="s">
-        <v>259</v>
       </c>
       <c r="G1" t="s">
         <v>103</v>
       </c>
       <c r="H1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -8165,13 +8152,13 @@
         <v>65</v>
       </c>
       <c r="E2" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F2" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F2" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -8190,13 +8177,13 @@
         <v>65</v>
       </c>
       <c r="E3" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F3" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F3" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -8215,13 +8202,13 @@
         <v>65</v>
       </c>
       <c r="E4" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F4" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F4" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -8240,13 +8227,13 @@
         <v>65</v>
       </c>
       <c r="E5" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F5" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F5" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -8265,13 +8252,13 @@
         <v>65</v>
       </c>
       <c r="E6" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F6" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F6" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H6" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -8290,13 +8277,13 @@
         <v>65</v>
       </c>
       <c r="E7" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F7" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F7" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -8315,13 +8302,13 @@
         <v>65</v>
       </c>
       <c r="E8" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F8" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F8" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H8" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -8340,13 +8327,13 @@
         <v>65</v>
       </c>
       <c r="E9" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F9" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F9" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -8365,13 +8352,13 @@
         <v>65</v>
       </c>
       <c r="E10" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F10" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F10" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H10" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
@@ -8390,13 +8377,13 @@
         <v>65</v>
       </c>
       <c r="E11" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F11" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F11" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -8415,13 +8402,13 @@
         <v>65</v>
       </c>
       <c r="E12" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F12" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F12" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -8440,13 +8427,13 @@
         <v>65</v>
       </c>
       <c r="E13" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F13" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F13" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
@@ -8465,13 +8452,13 @@
         <v>65</v>
       </c>
       <c r="E14" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F14" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F14" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -8490,13 +8477,13 @@
         <v>65</v>
       </c>
       <c r="E15" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F15" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F15" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -8515,13 +8502,13 @@
         <v>65</v>
       </c>
       <c r="E16" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F16" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F16" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H16" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -8540,13 +8527,13 @@
         <v>65</v>
       </c>
       <c r="E17" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F17" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F17" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H17" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
@@ -8565,13 +8552,13 @@
         <v>65</v>
       </c>
       <c r="E18" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F18" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F18" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H18" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
@@ -8590,13 +8577,13 @@
         <v>65</v>
       </c>
       <c r="E19" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F19" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F19" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H19" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
@@ -8615,13 +8602,13 @@
         <v>65</v>
       </c>
       <c r="E20" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F20" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F20" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H20" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
@@ -8640,13 +8627,13 @@
         <v>65</v>
       </c>
       <c r="E21" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F21" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F21" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H21" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
@@ -8665,13 +8652,13 @@
         <v>65</v>
       </c>
       <c r="E22" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F22" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F22" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H22" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
@@ -8690,13 +8677,13 @@
         <v>65</v>
       </c>
       <c r="E23" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F23" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F23" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H23" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
@@ -8715,13 +8702,13 @@
         <v>65</v>
       </c>
       <c r="E24" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F24" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F24" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H24" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
@@ -8740,13 +8727,13 @@
         <v>65</v>
       </c>
       <c r="E25" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F25" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F25" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H25" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
@@ -8765,13 +8752,13 @@
         <v>65</v>
       </c>
       <c r="E26" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F26" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F26" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H26" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
@@ -8790,13 +8777,13 @@
         <v>65</v>
       </c>
       <c r="E27" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F27" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F27" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H27" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
@@ -8815,13 +8802,13 @@
         <v>65</v>
       </c>
       <c r="E28" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F28" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F28" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H28" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
@@ -8840,13 +8827,13 @@
         <v>65</v>
       </c>
       <c r="E29" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F29" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F29" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H29" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
@@ -8865,13 +8852,13 @@
         <v>65</v>
       </c>
       <c r="E30" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F30" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F30" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H30" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
@@ -8890,13 +8877,13 @@
         <v>65</v>
       </c>
       <c r="E31" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F31" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F31" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H31" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
@@ -8915,13 +8902,13 @@
         <v>65</v>
       </c>
       <c r="E32" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F32" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F32" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H32" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.35">
@@ -8940,13 +8927,13 @@
         <v>65</v>
       </c>
       <c r="E33" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F33" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F33" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H33" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.35">
@@ -8965,13 +8952,13 @@
         <v>65</v>
       </c>
       <c r="E34" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F34" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F34" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H34" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.35">
@@ -8990,13 +8977,13 @@
         <v>65</v>
       </c>
       <c r="E35" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F35" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F35" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H35" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.35">
@@ -9015,13 +9002,13 @@
         <v>65</v>
       </c>
       <c r="E36" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F36" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F36" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.35">
@@ -9040,13 +9027,13 @@
         <v>65</v>
       </c>
       <c r="E37" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F37" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F37" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H37" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.35">
@@ -9065,13 +9052,13 @@
         <v>65</v>
       </c>
       <c r="E38" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F38" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F38" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.35">
@@ -9090,13 +9077,13 @@
         <v>65</v>
       </c>
       <c r="E39" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F39" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F39" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H39" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.35">
@@ -9115,13 +9102,13 @@
         <v>65</v>
       </c>
       <c r="E40" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F40" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F40" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H40" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.35">
@@ -9140,13 +9127,13 @@
         <v>65</v>
       </c>
       <c r="E41" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F41" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F41" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H41" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.35">
@@ -9165,13 +9152,13 @@
         <v>65</v>
       </c>
       <c r="E42" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F42" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F42" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H42" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R42" s="60"/>
       <c r="S42" s="60"/>
@@ -9192,13 +9179,13 @@
         <v>65</v>
       </c>
       <c r="E43" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F43" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F43" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H43" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R43" s="60"/>
       <c r="S43" s="60"/>
@@ -9219,13 +9206,13 @@
         <v>65</v>
       </c>
       <c r="E44" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F44" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F44" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H44" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R44" s="60"/>
       <c r="S44" s="60"/>
@@ -9246,13 +9233,13 @@
         <v>65</v>
       </c>
       <c r="E45" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F45" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F45" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H45" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R45" s="60"/>
       <c r="S45" s="60"/>
@@ -9273,13 +9260,13 @@
         <v>65</v>
       </c>
       <c r="E46" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F46" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F46" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H46" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R46" s="60"/>
       <c r="S46" s="60"/>
@@ -9300,13 +9287,13 @@
         <v>65</v>
       </c>
       <c r="E47" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F47" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F47" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H47" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R47" s="60"/>
       <c r="S47" s="60"/>
@@ -9327,13 +9314,13 @@
         <v>65</v>
       </c>
       <c r="E48" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F48" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F48" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H48" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R48" s="60"/>
       <c r="S48" s="60"/>
@@ -9354,13 +9341,13 @@
         <v>65</v>
       </c>
       <c r="E49" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F49" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F49" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H49" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R49" s="60"/>
       <c r="S49" s="60"/>
@@ -9381,13 +9368,13 @@
         <v>65</v>
       </c>
       <c r="E50" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F50" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F50" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H50" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R50" s="60"/>
       <c r="S50" s="60"/>
@@ -9408,13 +9395,13 @@
         <v>65</v>
       </c>
       <c r="E51" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F51" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F51" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H51" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R51" s="60"/>
       <c r="S51" s="60"/>
@@ -9435,13 +9422,13 @@
         <v>65</v>
       </c>
       <c r="E52" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F52" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F52" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H52" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R52" s="60"/>
       <c r="S52" s="60"/>
@@ -9462,13 +9449,13 @@
         <v>65</v>
       </c>
       <c r="E53" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F53" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F53" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H53" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R53" s="60"/>
       <c r="S53" s="60"/>
@@ -9489,13 +9476,13 @@
         <v>65</v>
       </c>
       <c r="E54" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F54" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F54" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H54" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.35">
@@ -9514,13 +9501,13 @@
         <v>65</v>
       </c>
       <c r="E55" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F55" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F55" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H55" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.35">
@@ -9539,13 +9526,13 @@
         <v>65</v>
       </c>
       <c r="E56" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F56" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F56" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H56" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.35">
@@ -9564,13 +9551,13 @@
         <v>65</v>
       </c>
       <c r="E57" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F57" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F57" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H57" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.35">
@@ -9589,13 +9576,13 @@
         <v>65</v>
       </c>
       <c r="E58" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F58" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F58" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H58" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.35">
@@ -9614,13 +9601,13 @@
         <v>65</v>
       </c>
       <c r="E59" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F59" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F59" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H59" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.35">
@@ -9639,13 +9626,13 @@
         <v>65</v>
       </c>
       <c r="E60" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F60" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F60" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H60" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.35">
@@ -9664,13 +9651,13 @@
         <v>65</v>
       </c>
       <c r="E61" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F61" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F61" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H61" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.35">
@@ -9689,13 +9676,13 @@
         <v>65</v>
       </c>
       <c r="E62" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F62" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F62" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H62" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.35">
@@ -9714,13 +9701,13 @@
         <v>65</v>
       </c>
       <c r="E63" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F63" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F63" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H63" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.35">
@@ -9739,13 +9726,13 @@
         <v>65</v>
       </c>
       <c r="E64" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F64" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F64" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H64" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.35">
@@ -9764,13 +9751,13 @@
         <v>65</v>
       </c>
       <c r="E65" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F65" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F65" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H65" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.35">
@@ -9789,13 +9776,13 @@
         <v>65</v>
       </c>
       <c r="E66" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F66" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F66" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H66" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.35">
@@ -9814,13 +9801,13 @@
         <v>65</v>
       </c>
       <c r="E67" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F67" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F67" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H67" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.35">
@@ -9839,13 +9826,13 @@
         <v>65</v>
       </c>
       <c r="E68" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F68" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F68" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H68" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.35">
@@ -9864,13 +9851,13 @@
         <v>65</v>
       </c>
       <c r="E69" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F69" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F69" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H69" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.35">
@@ -9889,13 +9876,13 @@
         <v>65</v>
       </c>
       <c r="E70" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F70" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F70" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H70" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.35">
@@ -9914,13 +9901,13 @@
         <v>65</v>
       </c>
       <c r="E71" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F71" s="60" t="s">
         <v>328</v>
       </c>
-      <c r="F71" s="60" t="s">
-        <v>329</v>
-      </c>
       <c r="H71" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.35">
@@ -9939,10 +9926,10 @@
         <v>65</v>
       </c>
       <c r="E72" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F72" s="60" t="s">
         <v>328</v>
-      </c>
-      <c r="F72" s="60" t="s">
-        <v>329</v>
       </c>
       <c r="H72" t="s">
         <v>115</v>
@@ -9964,10 +9951,10 @@
         <v>65</v>
       </c>
       <c r="E73" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F73" s="60" t="s">
         <v>328</v>
-      </c>
-      <c r="F73" s="60" t="s">
-        <v>329</v>
       </c>
       <c r="H73" t="s">
         <v>115</v>
@@ -9989,10 +9976,10 @@
         <v>65</v>
       </c>
       <c r="E74" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F74" s="60" t="s">
         <v>328</v>
-      </c>
-      <c r="F74" s="60" t="s">
-        <v>329</v>
       </c>
       <c r="H74" t="s">
         <v>115</v>
@@ -10014,10 +10001,10 @@
         <v>65</v>
       </c>
       <c r="E75" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F75" s="60" t="s">
         <v>328</v>
-      </c>
-      <c r="F75" s="60" t="s">
-        <v>329</v>
       </c>
       <c r="H75" t="s">
         <v>115</v>
@@ -10039,10 +10026,10 @@
         <v>65</v>
       </c>
       <c r="E76" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F76" s="60" t="s">
         <v>328</v>
-      </c>
-      <c r="F76" s="60" t="s">
-        <v>329</v>
       </c>
       <c r="H76" t="s">
         <v>115</v>
@@ -10064,10 +10051,10 @@
         <v>65</v>
       </c>
       <c r="E77" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F77" s="60" t="s">
         <v>328</v>
-      </c>
-      <c r="F77" s="60" t="s">
-        <v>329</v>
       </c>
       <c r="H77" t="s">
         <v>115</v>
@@ -10089,10 +10076,10 @@
         <v>65</v>
       </c>
       <c r="E78" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F78" s="60" t="s">
         <v>328</v>
-      </c>
-      <c r="F78" s="60" t="s">
-        <v>329</v>
       </c>
       <c r="H78" t="s">
         <v>115</v>
@@ -10114,10 +10101,10 @@
         <v>65</v>
       </c>
       <c r="E79" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F79" s="60" t="s">
         <v>328</v>
-      </c>
-      <c r="F79" s="60" t="s">
-        <v>329</v>
       </c>
       <c r="H79" t="s">
         <v>115</v>
@@ -10139,10 +10126,10 @@
         <v>65</v>
       </c>
       <c r="E80" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F80" s="60" t="s">
         <v>328</v>
-      </c>
-      <c r="F80" s="60" t="s">
-        <v>329</v>
       </c>
       <c r="H80" t="s">
         <v>115</v>
@@ -10164,10 +10151,10 @@
         <v>65</v>
       </c>
       <c r="E81" s="62" t="s">
+        <v>327</v>
+      </c>
+      <c r="F81" s="60" t="s">
         <v>328</v>
-      </c>
-      <c r="F81" s="60" t="s">
-        <v>329</v>
       </c>
       <c r="H81" t="s">
         <v>115</v>
@@ -10436,15 +10423,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B2">
         <v>0.24</v>
@@ -10492,7 +10479,7 @@
         <v>104</v>
       </c>
       <c r="C1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D1" t="s">
         <v>109</v>
@@ -10501,28 +10488,28 @@
         <v>110</v>
       </c>
       <c r="F1" t="s">
+        <v>176</v>
+      </c>
+      <c r="G1" t="s">
+        <v>182</v>
+      </c>
+      <c r="H1" t="s">
+        <v>197</v>
+      </c>
+      <c r="I1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J1" t="s">
         <v>177</v>
       </c>
-      <c r="G1" t="s">
-        <v>183</v>
-      </c>
-      <c r="H1" t="s">
-        <v>198</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>169</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>178</v>
       </c>
-      <c r="K1" t="s">
-        <v>170</v>
-      </c>
-      <c r="L1" t="s">
-        <v>179</v>
-      </c>
       <c r="M1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="N1" t="s">
         <v>111</v>
@@ -10531,19 +10518,19 @@
         <v>112</v>
       </c>
       <c r="P1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="Q1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="R1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="S1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="T1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.35">
@@ -10566,10 +10553,10 @@
         <v>79.5</v>
       </c>
       <c r="G2" s="60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H2" s="60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I2" s="37">
         <v>120</v>
@@ -10593,7 +10580,7 @@
         <v>42.2</v>
       </c>
       <c r="P2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T2" t="s">
         <v>114</v>
@@ -10619,10 +10606,10 @@
         <v>120</v>
       </c>
       <c r="G3" s="60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H3" s="60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I3">
         <v>287</v>
@@ -10646,7 +10633,7 @@
         <v>81.3</v>
       </c>
       <c r="P3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T3" t="s">
         <v>115</v>
@@ -10654,10 +10641,10 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" t="s">
         <v>166</v>
-      </c>
-      <c r="B4" t="s">
-        <v>167</v>
       </c>
       <c r="C4">
         <v>60</v>
@@ -10672,10 +10659,10 @@
         <v>29</v>
       </c>
       <c r="G4" s="60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H4" s="60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I4">
         <v>72</v>
@@ -10684,10 +10671,10 @@
         <v>105</v>
       </c>
       <c r="K4" s="60" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L4" s="60" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="M4">
         <v>200</v>
@@ -10699,7 +10686,7 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="P4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T4" t="s">
         <v>114</v>
@@ -10707,10 +10694,10 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>174</v>
+      </c>
+      <c r="B5" t="s">
         <v>175</v>
-      </c>
-      <c r="B5" t="s">
-        <v>176</v>
       </c>
       <c r="C5">
         <v>60</v>
@@ -10727,10 +10714,10 @@
         <v>31.5</v>
       </c>
       <c r="G5" s="60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H5" s="60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I5">
         <v>80.3</v>
@@ -10754,7 +10741,7 @@
         <v>6</v>
       </c>
       <c r="P5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T5" t="s">
         <v>115</v>
@@ -10762,10 +10749,10 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C6">
         <v>60</v>
@@ -10780,10 +10767,10 @@
         <v>43</v>
       </c>
       <c r="G6" s="60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H6" s="60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I6">
         <v>134</v>
@@ -10795,7 +10782,7 @@
         <v>23</v>
       </c>
       <c r="L6" s="60" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M6">
         <v>536</v>
@@ -10807,18 +10794,18 @@
         <v>5.4</v>
       </c>
       <c r="P6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C7">
         <v>60</v>
@@ -10848,7 +10835,7 @@
         <v>31</v>
       </c>
       <c r="L7" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="M7">
         <v>936</v>
@@ -10860,7 +10847,7 @@
         <v>9</v>
       </c>
       <c r="P7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T7" t="s">
         <v>115</v>
@@ -10868,10 +10855,10 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C8">
         <v>60</v>
@@ -10889,7 +10876,7 @@
         <v>53</v>
       </c>
       <c r="H8" s="60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I8">
         <v>100</v>
@@ -10901,7 +10888,7 @@
         <v>29</v>
       </c>
       <c r="L8" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="M8">
         <v>400</v>
@@ -10913,7 +10900,7 @@
         <v>3</v>
       </c>
       <c r="P8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="Q8">
         <v>4</v>
@@ -10941,10 +10928,10 @@
       <c r="K11" s="60"/>
       <c r="L11" s="60"/>
       <c r="N11" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O11" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.35">
@@ -11006,22 +10993,22 @@
         <v>103</v>
       </c>
       <c r="B1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E1" t="s">
         <v>282</v>
       </c>
-      <c r="E1" t="s">
-        <v>283</v>
-      </c>
       <c r="F1" t="s">
+        <v>275</v>
+      </c>
+      <c r="G1" t="s">
         <v>276</v>
-      </c>
-      <c r="G1" t="s">
-        <v>277</v>
       </c>
       <c r="H1" t="s">
         <v>133</v>
@@ -11316,10 +11303,10 @@
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B3" s="63"/>
-      <c r="C3" s="154" t="s">
+      <c r="C3" s="155" t="s">
         <v>117</v>
       </c>
-      <c r="D3" s="155"/>
+      <c r="D3" s="156"/>
       <c r="E3" s="64"/>
       <c r="G3" s="70" t="str">
         <f>C11</f>
@@ -11381,7 +11368,7 @@
         <v>1.25</v>
       </c>
       <c r="M4" s="73" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N4" s="85">
         <f>K15/(1-N3%)*N2</f>
@@ -11408,7 +11395,7 @@
       </c>
       <c r="E5" s="65"/>
       <c r="G5" s="70" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H5" s="61">
         <f>D23</f>
@@ -11423,7 +11410,7 @@
         <v>1.026</v>
       </c>
       <c r="M5" s="87" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="N5" s="88">
         <f>_xlfn.MINIFS(J21:J32,J21:J32,"&gt;="&amp;N4)</f>
@@ -11450,7 +11437,7 @@
       </c>
       <c r="E6" s="65"/>
       <c r="G6" s="87" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H6" s="89">
         <f>H2-H3-H4-H5</f>
@@ -11509,15 +11496,15 @@
     </row>
     <row r="8" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B8" s="63"/>
-      <c r="C8" s="154" t="s">
-        <v>205</v>
-      </c>
-      <c r="D8" s="155"/>
+      <c r="C8" s="155" t="s">
+        <v>204</v>
+      </c>
+      <c r="D8" s="156"/>
       <c r="E8" s="64"/>
       <c r="G8" s="75"/>
       <c r="H8" s="76"/>
       <c r="J8" s="87" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="K8" s="88">
         <f>K2+(K3+(K4+K5)*K6%)/K7*10^3</f>
@@ -11526,7 +11513,7 @@
       <c r="M8" s="75"/>
       <c r="N8" s="76"/>
       <c r="P8" s="87" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="Q8" s="105">
         <f>Q2-(Q2-Q3)*EXP(-Q4/Q5/Q6/(1-Q7%)*10^3)</f>
@@ -11536,7 +11523,7 @@
     <row r="9" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B9" s="63"/>
       <c r="C9" s="36" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D9" s="2" t="str">
         <f>HMI!E3</f>
@@ -11551,7 +11538,7 @@
     <row r="10" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B10" s="63"/>
       <c r="C10" s="36" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D10" s="7">
         <f>_xlfn.XLOOKUP(D9, DB_GD[Part], DB_GD[Vfint,100mA (V)])</f>
@@ -11620,7 +11607,7 @@
       </c>
       <c r="E12" s="65"/>
       <c r="G12" s="87" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H12" s="88">
         <f>H10-H11</f>
@@ -11665,7 +11652,7 @@
         <v>83.943749999999994</v>
       </c>
       <c r="M13" s="87" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="N13" s="105">
         <f>((1-N10%)/N11)*1000-N12/1000</f>
@@ -11724,7 +11711,7 @@
       </c>
       <c r="E15" s="65"/>
       <c r="J15" s="87" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="K15" s="88">
         <f>K13/K14</f>
@@ -11765,7 +11752,7 @@
       <c r="M16" s="75"/>
       <c r="N16" s="76"/>
       <c r="P16" s="87" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="Q16" s="88">
         <f>0.5*Q12*(1-Q13%)*Q14^2*Q15*10^-3</f>
@@ -11774,10 +11761,10 @@
     </row>
     <row r="17" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B17" s="63"/>
-      <c r="C17" s="154" t="s">
-        <v>213</v>
-      </c>
-      <c r="D17" s="155"/>
+      <c r="C17" s="155" t="s">
+        <v>212</v>
+      </c>
+      <c r="D17" s="156"/>
       <c r="E17" s="64"/>
       <c r="G17" s="70" t="str">
         <f>G5</f>
@@ -11804,7 +11791,7 @@
       </c>
       <c r="E18" s="65"/>
       <c r="G18" s="87" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H18" s="105">
         <f>H16-H17</f>
@@ -11858,12 +11845,12 @@
       <c r="E20" s="65"/>
       <c r="G20" s="75"/>
       <c r="H20" s="76"/>
-      <c r="J20" s="156" t="s">
-        <v>229</v>
-      </c>
-      <c r="K20" s="157"/>
+      <c r="J20" s="157" t="s">
+        <v>228</v>
+      </c>
+      <c r="K20" s="158"/>
       <c r="M20" s="87" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="N20" s="88">
         <f>N19*N18/(N18+N19)</f>
@@ -11880,15 +11867,15 @@
     </row>
     <row r="21" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B21" s="63"/>
-      <c r="C21" s="154" t="s">
-        <v>210</v>
-      </c>
-      <c r="D21" s="155"/>
+      <c r="C21" s="155" t="s">
+        <v>209</v>
+      </c>
+      <c r="D21" s="156"/>
       <c r="E21" s="64"/>
-      <c r="J21" s="140">
+      <c r="J21" s="151">
         <v>47</v>
       </c>
-      <c r="K21" s="141"/>
+      <c r="K21" s="152"/>
       <c r="M21" s="81"/>
       <c r="N21" s="82"/>
       <c r="P21" s="70" t="str">
@@ -11903,7 +11890,7 @@
     <row r="22" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B22" s="63"/>
       <c r="C22" s="36" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D22" s="2" t="str">
         <f>HMI!E8</f>
@@ -11918,10 +11905,10 @@
         <f>H18</f>
         <v>10.26</v>
       </c>
-      <c r="J22" s="140">
+      <c r="J22" s="151">
         <v>56</v>
       </c>
-      <c r="K22" s="141"/>
+      <c r="K22" s="152"/>
       <c r="M22" s="103"/>
       <c r="N22" s="104"/>
       <c r="P22" s="70" t="str">
@@ -11952,14 +11939,14 @@
         <f>D25</f>
         <v>10</v>
       </c>
-      <c r="J23" s="140">
+      <c r="J23" s="151">
         <v>68</v>
       </c>
-      <c r="K23" s="141"/>
+      <c r="K23" s="152"/>
       <c r="M23" s="75"/>
       <c r="N23" s="76"/>
       <c r="P23" s="87" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="Q23" s="105">
         <f>Q21/(Q20+Q21)*Q22</f>
@@ -11968,22 +11955,22 @@
     </row>
     <row r="24" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B24" s="63"/>
-      <c r="C24" s="154" t="s">
-        <v>216</v>
-      </c>
-      <c r="D24" s="155"/>
+      <c r="C24" s="155" t="s">
+        <v>215</v>
+      </c>
+      <c r="D24" s="156"/>
       <c r="E24" s="64"/>
       <c r="G24" s="87" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H24" s="105">
         <f>H22/H23</f>
         <v>1.026</v>
       </c>
-      <c r="J24" s="140">
+      <c r="J24" s="151">
         <v>82</v>
       </c>
-      <c r="K24" s="141"/>
+      <c r="K24" s="152"/>
       <c r="P24" s="81"/>
       <c r="Q24" s="82"/>
     </row>
@@ -12000,26 +11987,26 @@
       <c r="E25" s="65"/>
       <c r="G25" s="81"/>
       <c r="H25" s="82"/>
-      <c r="J25" s="140">
+      <c r="J25" s="151">
         <v>100</v>
       </c>
-      <c r="K25" s="141"/>
+      <c r="K25" s="152"/>
       <c r="P25" s="71"/>
       <c r="Q25" s="72"/>
     </row>
     <row r="26" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B26" s="63"/>
-      <c r="C26" s="154" t="s">
-        <v>226</v>
-      </c>
-      <c r="D26" s="155"/>
+      <c r="C26" s="155" t="s">
+        <v>225</v>
+      </c>
+      <c r="D26" s="156"/>
       <c r="E26" s="64"/>
       <c r="G26" s="75"/>
       <c r="H26" s="76"/>
-      <c r="J26" s="140">
+      <c r="J26" s="151">
         <v>120</v>
       </c>
-      <c r="K26" s="141"/>
+      <c r="K26" s="152"/>
       <c r="P26" s="75"/>
       <c r="Q26" s="76"/>
     </row>
@@ -12034,37 +12021,37 @@
         <v>3.3</v>
       </c>
       <c r="E27" s="65"/>
-      <c r="J27" s="140">
+      <c r="J27" s="151">
         <v>150</v>
       </c>
-      <c r="K27" s="141"/>
+      <c r="K27" s="152"/>
     </row>
     <row r="28" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B28" s="63"/>
-      <c r="C28" s="154" t="s">
+      <c r="C28" s="155" t="s">
         <v>102</v>
       </c>
-      <c r="D28" s="155"/>
+      <c r="D28" s="156"/>
       <c r="E28" s="64"/>
-      <c r="J28" s="140">
+      <c r="J28" s="151">
         <v>180</v>
       </c>
-      <c r="K28" s="141"/>
+      <c r="K28" s="152"/>
     </row>
     <row r="29" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B29" s="63"/>
       <c r="C29" s="36" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D29" s="2" t="str">
         <f>HMI!H4</f>
         <v>TI CSD18540Q5B</v>
       </c>
       <c r="E29" s="65"/>
-      <c r="J29" s="140">
+      <c r="J29" s="151">
         <v>220</v>
       </c>
-      <c r="K29" s="141"/>
+      <c r="K29" s="152"/>
     </row>
     <row r="30" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B30" s="63"/>
@@ -12077,29 +12064,37 @@
         <v>41</v>
       </c>
       <c r="E30" s="65"/>
-      <c r="J30" s="140">
+      <c r="J30" s="151">
         <v>470</v>
       </c>
-      <c r="K30" s="141"/>
+      <c r="K30" s="152"/>
     </row>
     <row r="31" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B31" s="63"/>
       <c r="C31" s="63"/>
       <c r="D31" s="63"/>
       <c r="E31" s="63"/>
-      <c r="J31" s="140">
+      <c r="J31" s="151">
         <v>680</v>
       </c>
-      <c r="K31" s="141"/>
+      <c r="K31" s="152"/>
     </row>
     <row r="32" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="J32" s="148">
+      <c r="J32" s="153">
         <v>1000</v>
       </c>
-      <c r="K32" s="149"/>
+      <c r="K32" s="154"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="J24:K24"/>
     <mergeCell ref="J25:K25"/>
@@ -12112,14 +12107,6 @@
     <mergeCell ref="C26:D26"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="C21:D21"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12167,10 +12154,10 @@
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B3" s="63"/>
-      <c r="C3" s="154" t="s">
+      <c r="C3" s="155" t="s">
         <v>117</v>
       </c>
-      <c r="D3" s="155"/>
+      <c r="D3" s="156"/>
       <c r="E3" s="64"/>
       <c r="G3" s="70" t="str">
         <f>C7</f>
@@ -12232,7 +12219,7 @@
       </c>
       <c r="E6" s="65"/>
       <c r="G6" s="73" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H6" s="85">
         <f>H2^2*H4*H5%</f>
@@ -12251,7 +12238,7 @@
       </c>
       <c r="E7" s="65"/>
       <c r="G7" s="87" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H7" s="88">
         <f>H3^2*H4*H5%</f>
@@ -12302,11 +12289,11 @@
     </row>
     <row r="11" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B11" s="63"/>
-      <c r="C11" s="154" t="str">
+      <c r="C11" s="155" t="str">
         <f>HMI!H2</f>
         <v>MOSFET</v>
       </c>
-      <c r="D11" s="155"/>
+      <c r="D11" s="156"/>
       <c r="E11" s="65"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.35">
@@ -12351,10 +12338,10 @@
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B14" s="63"/>
-      <c r="C14" s="154" t="s">
-        <v>309</v>
-      </c>
-      <c r="D14" s="155"/>
+      <c r="C14" s="155" t="s">
+        <v>308</v>
+      </c>
+      <c r="D14" s="156"/>
       <c r="E14" s="65"/>
       <c r="G14" s="70" t="str">
         <f>C7</f>
@@ -12421,7 +12408,7 @@
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.35">
       <c r="G18" s="73" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H18" s="85">
         <f>0.5*H12*H13*H15*(H16+H17)*10^-3</f>
@@ -12430,7 +12417,7 @@
     </row>
     <row r="19" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="G19" s="73" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H19" s="85">
         <f>0.5*H12*H14*H15*(H16+H17)*10^-3</f>
@@ -12492,7 +12479,7 @@
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.35">
       <c r="G28" s="73" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H28" s="85">
         <f>2*H24+4*H26</f>
@@ -12501,7 +12488,7 @@
     </row>
     <row r="29" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="G29" s="73" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H29" s="88">
         <f>2*H25+4*H27</f>
@@ -12602,10 +12589,10 @@
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B3" s="63"/>
-      <c r="C3" s="154" t="s">
+      <c r="C3" s="155" t="s">
         <v>117</v>
       </c>
-      <c r="D3" s="155"/>
+      <c r="D3" s="156"/>
       <c r="E3" s="65"/>
       <c r="G3" s="70" t="str">
         <f>C9</f>
@@ -12651,7 +12638,7 @@
       </c>
       <c r="E4" s="65"/>
       <c r="G4" s="79" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H4" s="83">
         <f>H2*H3/(H3+H2)</f>
@@ -12693,24 +12680,24 @@
         <v>90</v>
       </c>
       <c r="E5" s="63"/>
-      <c r="G5" s="158"/>
-      <c r="H5" s="159"/>
+      <c r="G5" s="159"/>
+      <c r="H5" s="160"/>
       <c r="J5" s="73" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="K5" s="74">
         <f>K2/K3</f>
         <v>1.7389830508474575</v>
       </c>
       <c r="M5" s="87" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="N5" s="89">
         <f>N2*N3*N4*10^-3</f>
         <v>26.922239999999999</v>
       </c>
       <c r="P5" s="79" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="Q5" s="86">
         <f>Q4*Q2/(Q2+Q3)</f>
@@ -12728,33 +12715,33 @@
         <v>64</v>
       </c>
       <c r="E6" s="64"/>
-      <c r="G6" s="160"/>
-      <c r="H6" s="161"/>
+      <c r="G6" s="161"/>
+      <c r="H6" s="162"/>
       <c r="J6" s="87" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K6" s="105">
         <f>K2/K4</f>
         <v>2.2768614691527969</v>
       </c>
-      <c r="M6" s="158"/>
-      <c r="N6" s="159"/>
+      <c r="M6" s="159"/>
+      <c r="N6" s="160"/>
       <c r="P6" s="95"/>
       <c r="Q6" s="96"/>
     </row>
     <row r="7" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B7" s="63"/>
-      <c r="C7" s="154" t="s">
-        <v>231</v>
-      </c>
-      <c r="D7" s="155"/>
+      <c r="C7" s="155" t="s">
+        <v>230</v>
+      </c>
+      <c r="D7" s="156"/>
       <c r="E7" s="65"/>
-      <c r="G7" s="162"/>
-      <c r="H7" s="163"/>
+      <c r="G7" s="163"/>
+      <c r="H7" s="164"/>
       <c r="J7" s="71"/>
       <c r="K7" s="72"/>
-      <c r="M7" s="162"/>
-      <c r="N7" s="163"/>
+      <c r="M7" s="163"/>
+      <c r="N7" s="164"/>
       <c r="P7" s="97"/>
       <c r="Q7" s="98"/>
     </row>
@@ -12806,10 +12793,10 @@
     </row>
     <row r="10" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B10" s="63"/>
-      <c r="C10" s="154" t="s">
-        <v>232</v>
-      </c>
-      <c r="D10" s="155"/>
+      <c r="C10" s="155" t="s">
+        <v>231</v>
+      </c>
+      <c r="D10" s="156"/>
       <c r="E10" s="64"/>
       <c r="G10" s="70" t="str">
         <f>C13</f>
@@ -12841,7 +12828,7 @@
     <row r="11" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B11" s="63"/>
       <c r="C11" s="36" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D11" s="2" t="str">
         <f>HMI!E3</f>
@@ -12857,7 +12844,7 @@
         <v>3.3</v>
       </c>
       <c r="M11" s="87" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="N11" s="88">
         <f>N9*N10</f>
@@ -12899,8 +12886,8 @@
         <f>D23</f>
         <v>4</v>
       </c>
-      <c r="M12" s="164"/>
-      <c r="N12" s="165"/>
+      <c r="M12" s="165"/>
+      <c r="N12" s="166"/>
       <c r="P12" s="70" t="str">
         <f>P5</f>
         <v>Prg,mean (mW)</v>
@@ -12922,7 +12909,7 @@
       </c>
       <c r="E13" s="65"/>
       <c r="G13" s="79" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H13" s="83">
         <f>(H10+H9)/2+H11+H12</f>
@@ -12936,10 +12923,10 @@
         <f>H13</f>
         <v>5.9</v>
       </c>
-      <c r="M13" s="166"/>
-      <c r="N13" s="167"/>
+      <c r="M13" s="167"/>
+      <c r="N13" s="168"/>
       <c r="P13" s="79" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="Q13" s="83">
         <f>0.5*(1+Q10/(Q10+Q11))*Q12</f>
@@ -12984,7 +12971,7 @@
       <c r="G15" s="109"/>
       <c r="H15" s="110"/>
       <c r="J15" s="73" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K15" s="74">
         <f>K12/K13</f>
@@ -13015,7 +13002,7 @@
       <c r="G16" s="111"/>
       <c r="H16" s="112"/>
       <c r="J16" s="87" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="K16" s="105">
         <f>K12/K14</f>
@@ -13094,10 +13081,10 @@
     </row>
     <row r="19" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B19" s="63"/>
-      <c r="C19" s="154" t="s">
+      <c r="C19" s="155" t="s">
         <v>102</v>
       </c>
-      <c r="D19" s="155"/>
+      <c r="D19" s="156"/>
       <c r="E19" s="63"/>
       <c r="G19" s="70" t="str">
         <f>C15</f>
@@ -13129,7 +13116,7 @@
     <row r="20" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B20" s="63"/>
       <c r="C20" s="36" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D20" s="2" t="str">
         <f>HMI!H4</f>
@@ -13147,14 +13134,14 @@
       <c r="J20" s="75"/>
       <c r="K20" s="76"/>
       <c r="M20" s="87" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="N20" s="89">
         <f>(N15%*(N17+N16)+(1-N15%)*(N18+N19))/4</f>
         <v>0.47125</v>
       </c>
       <c r="P20" s="79" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="Q20" s="89">
         <f>Q18-Q19</f>
@@ -13180,8 +13167,8 @@
         <f>D24</f>
         <v>1.6</v>
       </c>
-      <c r="M21" s="158"/>
-      <c r="N21" s="159"/>
+      <c r="M21" s="159"/>
+      <c r="N21" s="160"/>
       <c r="P21" s="107"/>
       <c r="Q21" s="108"/>
     </row>
@@ -13197,7 +13184,7 @@
       </c>
       <c r="E22" s="64"/>
       <c r="G22" s="79" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H22" s="83">
         <f>(H18+H19)/2+H20+H21</f>
@@ -13211,8 +13198,8 @@
         <f>D22</f>
         <v>6.7</v>
       </c>
-      <c r="M22" s="160"/>
-      <c r="N22" s="161"/>
+      <c r="M22" s="161"/>
+      <c r="N22" s="162"/>
       <c r="P22" s="111"/>
       <c r="Q22" s="112"/>
     </row>
@@ -13237,8 +13224,8 @@
         <f>K15</f>
         <v>0.67796610169491522</v>
       </c>
-      <c r="M23" s="162"/>
-      <c r="N23" s="163"/>
+      <c r="M23" s="163"/>
+      <c r="N23" s="164"/>
     </row>
     <row r="24" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B24" s="63"/>
@@ -13278,7 +13265,7 @@
       <c r="G25" s="111"/>
       <c r="H25" s="112"/>
       <c r="J25" s="73" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="K25" s="74">
         <f>K22/K23</f>
@@ -13303,7 +13290,7 @@
     </row>
     <row r="26" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="J26" s="87" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K26" s="105">
         <f>K22/K24</f>
@@ -13318,7 +13305,7 @@
         <v>3.3</v>
       </c>
       <c r="P26" s="87" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="Q26" s="88">
         <f>Q24-Q25</f>
@@ -13343,7 +13330,7 @@
       <c r="J28" s="71"/>
       <c r="K28" s="72"/>
       <c r="M28" s="87" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="N28" s="89">
         <f>(N25%*N26+(1-N25%)*N27)/2</f>
@@ -13413,18 +13400,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B2" s="171" t="s">
+      <c r="B2" s="172" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="172"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
-      <c r="F2" s="172"/>
-      <c r="G2" s="172"/>
-      <c r="H2" s="172"/>
-      <c r="I2" s="172"/>
-      <c r="J2" s="172"/>
-      <c r="K2" s="173"/>
+      <c r="C2" s="173"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
+      <c r="F2" s="173"/>
+      <c r="G2" s="173"/>
+      <c r="H2" s="173"/>
+      <c r="I2" s="173"/>
+      <c r="J2" s="173"/>
+      <c r="K2" s="174"/>
       <c r="M2" s="8" t="str">
         <f>HMI!B13</f>
         <v>Vph spike (V) @ disarm</v>
@@ -13887,7 +13874,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="M10" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="N10" s="2">
         <f>HMI!C7</f>
@@ -14373,11 +14360,11 @@
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="M19" s="168" t="s">
+      <c r="M19" s="169" t="s">
         <v>23</v>
       </c>
-      <c r="N19" s="169"/>
-      <c r="O19" s="170"/>
+      <c r="N19" s="170"/>
+      <c r="O19" s="171"/>
       <c r="Q19" t="s">
         <v>20</v>
       </c>
@@ -15237,7 +15224,7 @@
       </c>
       <c r="H2" s="69">
         <f>D11</f>
-        <v>850</v>
+        <v>500</v>
       </c>
       <c r="J2" s="68" t="str">
         <f>C16</f>
@@ -15250,10 +15237,10 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B3" s="63"/>
-      <c r="C3" s="154" t="s">
+      <c r="C3" s="155" t="s">
         <v>117</v>
       </c>
-      <c r="D3" s="155"/>
+      <c r="D3" s="156"/>
       <c r="E3" s="64"/>
       <c r="G3" s="70" t="str">
         <f>C5</f>
@@ -15283,11 +15270,11 @@
       </c>
       <c r="E4" s="65"/>
       <c r="G4" s="87" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H4" s="88">
         <f>H3*H2/1000</f>
-        <v>10.625</v>
+        <v>6.25</v>
       </c>
       <c r="J4" s="70" t="str">
         <f>G9</f>
@@ -15317,7 +15304,7 @@
       </c>
       <c r="K5" s="61">
         <f>D11</f>
-        <v>850</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -15334,11 +15321,11 @@
       <c r="G6" s="75"/>
       <c r="H6" s="76"/>
       <c r="J6" s="87" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="K6" s="89">
         <f>K2/(2^K3-1)/K4/K5*10^9</f>
-        <v>14.813617754794226</v>
+        <v>25.183150183150182</v>
       </c>
     </row>
     <row r="7" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -15372,7 +15359,7 @@
       </c>
       <c r="H8" s="69">
         <f>H4</f>
-        <v>10.625</v>
+        <v>6.25</v>
       </c>
       <c r="J8" s="103"/>
       <c r="K8" s="104"/>
@@ -15401,28 +15388,28 @@
     </row>
     <row r="10" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B10" s="63"/>
-      <c r="C10" s="154" t="s">
-        <v>242</v>
-      </c>
-      <c r="D10" s="155"/>
+      <c r="C10" s="155" t="s">
+        <v>241</v>
+      </c>
+      <c r="D10" s="156"/>
       <c r="E10" s="63"/>
       <c r="G10" s="87" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H10" s="88">
         <f>H9*H8/1000</f>
-        <v>0.68</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B11" s="63"/>
       <c r="C11" s="36" t="str">
-        <f>HMI!K4</f>
+        <f>HMI!K7</f>
         <v>Rshunt (µΩ)</v>
       </c>
       <c r="D11" s="2">
-        <f>HMI!L4</f>
-        <v>850</v>
+        <f>HMI!L7</f>
+        <v>500</v>
       </c>
       <c r="E11" s="64"/>
       <c r="G11" s="81"/>
@@ -15433,15 +15420,15 @@
       </c>
       <c r="K11" s="69">
         <f>D11</f>
-        <v>850</v>
+        <v>500</v>
       </c>
     </row>
     <row r="12" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="63"/>
-      <c r="C12" s="154" t="s">
-        <v>246</v>
-      </c>
-      <c r="D12" s="155"/>
+      <c r="C12" s="155" t="s">
+        <v>245</v>
+      </c>
+      <c r="D12" s="156"/>
       <c r="E12" s="64"/>
       <c r="G12" s="75"/>
       <c r="H12" s="76"/>
@@ -15461,7 +15448,7 @@
         <v>Name</v>
       </c>
       <c r="D13" s="2" t="str">
-        <f>HMI!K8</f>
+        <f>HMI!K4</f>
         <v>STM32G4 internal</v>
       </c>
       <c r="E13" s="64"/>
@@ -15477,11 +15464,11 @@
     <row r="14" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B14" s="63"/>
       <c r="C14" s="36" t="str">
-        <f>HMI!K11</f>
+        <f>HMI!K8</f>
         <v>Resolution (bit)</v>
       </c>
       <c r="D14" s="2">
-        <f>HMI!L11</f>
+        <f>HMI!L8</f>
         <v>12</v>
       </c>
       <c r="E14" s="64"/>
@@ -15494,21 +15481,21 @@
         <v>50</v>
       </c>
       <c r="J14" s="79" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="K14" s="86">
         <f>K11/10^3*K12^2*K13%*2/3</f>
-        <v>84.934902750000006</v>
+        <v>49.961707500000017</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B15" s="63"/>
       <c r="C15" s="36" t="str">
-        <f>HMI!K13</f>
+        <f>HMI!K10</f>
         <v>OpAmp gain</v>
       </c>
       <c r="D15" s="2">
-        <f>HMI!L13</f>
+        <f>HMI!L10</f>
         <v>64</v>
       </c>
       <c r="E15" s="64"/>
@@ -15518,7 +15505,7 @@
       </c>
       <c r="H15" s="61">
         <f>D11</f>
-        <v>850</v>
+        <v>500</v>
       </c>
       <c r="J15" s="81"/>
       <c r="K15" s="82"/>
@@ -15535,11 +15522,11 @@
       </c>
       <c r="E16" s="64"/>
       <c r="G16" s="87" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H16" s="88">
         <f>H15*H14/1000</f>
-        <v>42.5</v>
+        <v>25</v>
       </c>
       <c r="J16" s="71"/>
       <c r="K16" s="72"/>
@@ -15569,7 +15556,7 @@
       </c>
       <c r="K19" s="69">
         <f>K11</f>
-        <v>850</v>
+        <v>500</v>
       </c>
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.35">
@@ -15581,7 +15568,7 @@
       </c>
       <c r="H20" s="69">
         <f>H16</f>
-        <v>42.5</v>
+        <v>25</v>
       </c>
       <c r="J20" s="70" t="str">
         <f>C6</f>
@@ -15616,18 +15603,18 @@
       <c r="B22" s="64"/>
       <c r="E22" s="64"/>
       <c r="G22" s="87" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H22" s="88">
         <f>H21*H20/1000</f>
-        <v>2.72</v>
+        <v>1.6</v>
       </c>
       <c r="J22" s="79" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="K22" s="86">
         <f>K19/10^3*K20^2*K21%*2/3</f>
-        <v>204</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.35">
@@ -15684,14 +15671,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B2" s="174" t="s">
+      <c r="B2" s="175" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="174"/>
-      <c r="D2" s="174"/>
-      <c r="E2" s="174"/>
-      <c r="F2" s="174"/>
-      <c r="G2" s="174"/>
+      <c r="C2" s="175"/>
+      <c r="D2" s="175"/>
+      <c r="E2" s="175"/>
+      <c r="F2" s="175"/>
+      <c r="G2" s="175"/>
       <c r="I2" s="8" t="s">
         <v>48</v>
       </c>
@@ -15710,13 +15697,13 @@
         <v>53</v>
       </c>
       <c r="D3" s="52" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E3" s="52" t="s">
+        <v>157</v>
+      </c>
+      <c r="F3" s="53" t="s">
         <v>158</v>
-      </c>
-      <c r="F3" s="53" t="s">
-        <v>159</v>
       </c>
       <c r="G3" s="53" t="s">
         <v>59</v>
@@ -16185,10 +16172,10 @@
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B3" s="63"/>
-      <c r="C3" s="154" t="s">
+      <c r="C3" s="155" t="s">
         <v>117</v>
       </c>
-      <c r="D3" s="155"/>
+      <c r="D3" s="156"/>
       <c r="E3" s="64"/>
       <c r="G3" s="70" t="str">
         <f>C5</f>
@@ -16250,7 +16237,7 @@
         <v>1000</v>
       </c>
       <c r="M4" s="87" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="N4" s="88">
         <f>N2*N3/(N3+N2)</f>
@@ -16277,14 +16264,14 @@
       </c>
       <c r="E5" s="65"/>
       <c r="G5" s="73" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H5" s="85">
         <f>H2*(H3/H4-1)</f>
         <v>9606.0606060606078</v>
       </c>
       <c r="J5" s="79" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="K5" s="80">
         <f>K2/(K3+K4)*10^3</f>
@@ -16293,7 +16280,7 @@
       <c r="M5" s="81"/>
       <c r="N5" s="82"/>
       <c r="P5" s="79" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="Q5" s="83">
         <f>Q4+Q3+Q2</f>
@@ -16312,7 +16299,7 @@
       </c>
       <c r="E6" s="65"/>
       <c r="G6" s="79" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H6" s="86">
         <f>_xlfn.MINIFS(DB_R[R (Ω)],DB_R[R (Ω)],"&gt;="&amp;H5)</f>
@@ -16327,10 +16314,10 @@
     </row>
     <row r="7" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B7" s="63"/>
-      <c r="C7" s="154" t="s">
-        <v>246</v>
-      </c>
-      <c r="D7" s="155"/>
+      <c r="C7" s="155" t="s">
+        <v>245</v>
+      </c>
+      <c r="D7" s="156"/>
       <c r="E7" s="63"/>
       <c r="G7" s="81"/>
       <c r="H7" s="82"/>
@@ -16513,7 +16500,7 @@
         <v>35</v>
       </c>
       <c r="J13" s="73" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="K13" s="85">
         <f>K10/K12*1000</f>
@@ -16528,7 +16515,7 @@
         <v>33</v>
       </c>
       <c r="P13" s="79" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="Q13" s="83">
         <f>Q9*(Q10+Q11)*(Q12)*10^-3</f>
@@ -16547,14 +16534,14 @@
       </c>
       <c r="E14" s="63"/>
       <c r="G14" s="79" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="H14" s="86">
         <f>H13^2/(H11+H12)*1000</f>
         <v>111.36363636363636</v>
       </c>
       <c r="J14" s="79" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="K14" s="86">
         <f>K11/K12*1000</f>
@@ -16587,7 +16574,7 @@
       <c r="J15" s="81"/>
       <c r="K15" s="82"/>
       <c r="M15" s="79" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="N15" s="83">
         <f>1/2/PI()/(N12+N13)/N14/10^-6</f>
@@ -16598,11 +16585,11 @@
     </row>
     <row r="16" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B16" s="64"/>
-      <c r="C16" s="154" t="str">
+      <c r="C16" s="155" t="str">
         <f>HMI!N2</f>
         <v>Rv2 &amp; Rtrace</v>
       </c>
-      <c r="D16" s="155"/>
+      <c r="D16" s="156"/>
       <c r="E16" s="64"/>
       <c r="G16" s="71"/>
       <c r="H16" s="72"/>
@@ -16634,7 +16621,7 @@
     <row r="18" spans="2:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B18" s="63"/>
       <c r="C18" s="36" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D18" s="2">
         <f>_xlfn.XLOOKUP(D17, DB_R[Description], DB_R[R (Ω)])</f>
@@ -16671,7 +16658,7 @@
     <row r="20" spans="2:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B20" s="63"/>
       <c r="C20" s="36" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D20" s="2">
         <f>_xlfn.XLOOKUP(D19, DB_R[Description], DB_R[R (Ω)])</f>
@@ -16697,10 +16684,10 @@
     </row>
     <row r="21" spans="2:25" x14ac:dyDescent="0.35">
       <c r="B21" s="63"/>
-      <c r="C21" s="154" t="s">
-        <v>265</v>
-      </c>
-      <c r="D21" s="155"/>
+      <c r="C21" s="155" t="s">
+        <v>264</v>
+      </c>
+      <c r="D21" s="156"/>
       <c r="E21" s="65"/>
       <c r="G21" s="70" t="str">
         <f>C5</f>
@@ -16757,7 +16744,7 @@
         <v>3.3</v>
       </c>
       <c r="M22" s="87" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="N22" s="88">
         <f>N20*(1-N21%)</f>
@@ -16778,7 +16765,7 @@
       </c>
       <c r="E23" s="65"/>
       <c r="G23" s="73" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="H23" s="74">
         <f>H20*H21/(H20+H19)</f>
@@ -16809,7 +16796,7 @@
       </c>
       <c r="E24" s="65"/>
       <c r="G24" s="79" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H24" s="80">
         <f>H20*H22/(H20+H19)</f>
@@ -16842,7 +16829,7 @@
       <c r="G25" s="81"/>
       <c r="H25" s="82"/>
       <c r="J25" s="79" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K25" s="83">
         <f>K22/K21/(2^K23-1)*K24*1000</f>
@@ -16923,7 +16910,7 @@
       <c r="B30" s="63"/>
       <c r="E30" s="63"/>
       <c r="M30" s="79" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="N30" s="83">
         <f>N26*(N27+N28)*N29*10^-3</f>
@@ -17020,10 +17007,10 @@
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B3" s="63"/>
-      <c r="C3" s="154" t="s">
+      <c r="C3" s="155" t="s">
         <v>117</v>
       </c>
-      <c r="D3" s="155"/>
+      <c r="D3" s="156"/>
       <c r="E3" s="64"/>
       <c r="G3" s="70" t="str">
         <f>C11</f>
@@ -17065,7 +17052,7 @@
       </c>
       <c r="E5" s="65"/>
       <c r="G5" s="87" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="H5" s="105">
         <f>H3/(H2+H3)*H4</f>
@@ -17088,10 +17075,10 @@
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B7" s="63"/>
-      <c r="C7" s="154" t="s">
-        <v>327</v>
-      </c>
-      <c r="D7" s="155"/>
+      <c r="C7" s="155" t="s">
+        <v>326</v>
+      </c>
+      <c r="D7" s="156"/>
       <c r="E7" s="65"/>
       <c r="G7" s="71"/>
       <c r="H7" s="72"/>
@@ -17113,7 +17100,7 @@
     <row r="9" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B9" s="63"/>
       <c r="C9" s="36" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D9" s="2">
         <f>_xlfn.XLOOKUP(D8, DB_R[Description], DB_R[R (Ω)])</f>
@@ -17143,10 +17130,10 @@
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B11" s="63"/>
-      <c r="C11" s="175" t="s">
-        <v>334</v>
-      </c>
-      <c r="D11" s="176">
+      <c r="C11" s="137" t="s">
+        <v>333</v>
+      </c>
+      <c r="D11" s="1">
         <f>_xlfn.XLOOKUP(D10, DB_R[Description], DB_R[R (Ω)])</f>
         <v>1000</v>
       </c>
@@ -17176,7 +17163,7 @@
     </row>
     <row r="13" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="G13" s="87" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H13" s="105">
         <f>H11/(H10+H11)*H12</f>
@@ -17218,7 +17205,7 @@
     </row>
     <row r="20" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="G20" s="87" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H20" s="105">
         <f>(H18*H19)/(H18+H19)</f>

</xml_diff>